<commit_message>
docs: registrar integracion local y revision conjunta A B C
</commit_message>
<xml_diff>
--- a/docs/seguimiento/01_Seguimiento_Tsung_Hao_Fase2.xlsx
+++ b/docs/seguimiento/01_Seguimiento_Tsung_Hao_Fase2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloque A" sheetId="1" r:id="R785936381e0f418f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pruebas" sheetId="2" r:id="R05130be33cda4f39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rúbrica" sheetId="3" r:id="Rfb18e2580a654ae3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendientes" sheetId="4" r:id="Red2b9566c84841a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloque A" sheetId="1" r:id="Rbe139a5e1b0f44b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pruebas" sheetId="2" r:id="Re9ab2ebef5424fb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rúbrica" sheetId="3" r:id="Rbdb294ec03f2446f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendientes" sheetId="4" r:id="Rffd17e2c5a15456c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -97,7 +97,7 @@
         <x:color rgb="FFA12218"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE9E7"/>
         </x:patternFill>
       </x:fill>
@@ -312,7 +312,7 @@
   <x:sheetData>
     <x:row r="2">
       <x:c r="A2" s="1" t="str">
-        <x:v>Seguimiento de Tsung-Hao al 29 de septiembre de 2026</x:v>
+        <x:v>Seguimiento de Tsung-Hao al 20 de octubre de 2026</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
@@ -637,7 +637,7 @@
   <x:sheetData>
     <x:row r="2">
       <x:c r="A2" s="1" t="str">
-        <x:v>Resultados reproducibles en Docker local</x:v>
+        <x:v>Regresión A y común del 20/10. Resultados completos A/B/C en guía 04.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
@@ -665,10 +665,10 @@
         <x:v>unit</x:v>
       </x:c>
       <x:c r="B6" s="4" t="n">
-        <x:v>5</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C6" s="4" t="n">
-        <x:v>5</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D6" s="4" t="n">
         <x:v>0</x:v>
@@ -678,7 +678,7 @@
         <x:v>Sin fallos</x:v>
       </x:c>
       <x:c r="F6" s="4" t="str">
-        <x:v>../evidencias/equipo-a/unit.txt</x:v>
+        <x:v>../evidencias/integracion/final-unit.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
@@ -699,7 +699,7 @@
         <x:v>Sin fallos</x:v>
       </x:c>
       <x:c r="F7" s="4" t="str">
-        <x:v>../evidencias/equipo-a/a-sprint1.txt</x:v>
+        <x:v>../evidencias/integracion/final-a-sprint1.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
@@ -720,7 +720,7 @@
         <x:v>Sin fallos</x:v>
       </x:c>
       <x:c r="F8" s="4" t="str">
-        <x:v>../evidencias/equipo-a/a-sprint2.txt</x:v>
+        <x:v>../evidencias/integracion/final-a-sprint2.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
@@ -741,12 +741,12 @@
         <x:v>Sin fallos</x:v>
       </x:c>
       <x:c r="F9" s="4" t="str">
-        <x:v>../evidencias/equipo-a/a-ops.txt</x:v>
+        <x:v>../evidencias/integracion/final-a-ops.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
       <x:c r="A10" s="4" t="str">
-        <x:v>smoke-base</x:v>
+        <x:v>smoke</x:v>
       </x:c>
       <x:c r="B10" s="4" t="n">
         <x:v>7</x:v>
@@ -762,18 +762,18 @@
         <x:v>Sin fallos</x:v>
       </x:c>
       <x:c r="F10" s="4" t="str">
-        <x:v>../evidencias/equipo-a/smoke-base.txt</x:v>
+        <x:v>../evidencias/integracion/final-smoke.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
       <x:c r="A11" s="4" t="str">
-        <x:v>smoke-ops</x:v>
+        <x:v>frontend-unit</x:v>
       </x:c>
       <x:c r="B11" s="4" t="n">
-        <x:v>7</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C11" s="4" t="n">
-        <x:v>7</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D11" s="4" t="n">
         <x:v>0</x:v>
@@ -783,7 +783,7 @@
         <x:v>Sin fallos</x:v>
       </x:c>
       <x:c r="F11" s="4" t="str">
-        <x:v>../evidencias/equipo-a/smoke-ops.txt</x:v>
+        <x:v>../evidencias/integracion/final-frontend-unit.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -794,17 +794,17 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C12" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D12" s="4" t="n">
-        <x:v>7</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E12" s="4" t="str">
         <x:f>IF(D12&gt;0,"Con fallos","Sin fallos")</x:f>
-        <x:v>Con fallos</x:v>
+        <x:v>Sin fallos</x:v>
       </x:c>
       <x:c r="F12" s="4" t="str">
-        <x:v>../evidencias/equipo-a/contract.txt</x:v>
+        <x:v>../evidencias/integracion/final-contract.txt</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1048,7 +1048,7 @@
         <x:v>Cumplimiento técnico</x:v>
       </x:c>
       <x:c r="E15" s="4" t="str">
-        <x:v>Evidencia local A</x:v>
+        <x:v>Regresión conjunta A/B/C en Docker</x:v>
       </x:c>
       <x:c r="F15" s="4" t="str">
         <x:v>B/C e integración pendientes</x:v>
@@ -1364,16 +1364,16 @@
         <x:v>A-06</x:v>
       </x:c>
       <x:c r="B11" s="4" t="str">
-        <x:v>7 defectos contractuales B/C</x:v>
+        <x:v>Ocho detectores contractuales aprobados</x:v>
       </x:c>
       <x:c r="C11" s="4" t="str">
-        <x:v>Corregir sin borrar ni omitir las pruebas</x:v>
+        <x:v>Corregir note en E18 y validar Stripe real; ver guía 04</x:v>
       </x:c>
       <x:c r="D11" s="4" t="str">
         <x:v>Catalina / Felipe</x:v>
       </x:c>
       <x:c r="E11" s="4" t="str">
-        <x:v>Abierto</x:v>
+        <x:v>Pendientes puntuales</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -1432,16 +1432,16 @@
         <x:v>A-10</x:v>
       </x:c>
       <x:c r="B15" s="4" t="str">
-        <x:v>No hay publicación nueva</x:v>
+        <x:v>Integración local de A/B/C preparada</x:v>
       </x:c>
       <x:c r="C15" s="4" t="str">
-        <x:v>Solicitar revisión y autorización antes de push o despliegue</x:v>
+        <x:v>Revisar antes de autorizar publicación de la rama integrada</x:v>
       </x:c>
       <x:c r="D15" s="4" t="str">
         <x:v>Tsung-Hao</x:v>
       </x:c>
       <x:c r="E15" s="4" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Sin push nuevo</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>